<commit_message>
fixed sch according to last DR
</commit_message>
<xml_diff>
--- a/MIB_components.xlsx
+++ b/MIB_components.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arian\Documents\RAMMP\repos\RAMMP-Electronics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E25266B-BA61-4D0E-AE3C-70C929B8A040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{428DDCC4-4630-4A5B-929E-6F6C5B33DFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{6F4A9416-ED2C-4136-AA62-A972BF68C866}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="136">
   <si>
     <t>Digikey link</t>
   </si>
@@ -58,27 +58,7 @@
     <t>JLC part #</t>
   </si>
   <si>
-    <t>https://jlcpcb.com/partdetail/TexasInstruments-INA118PB/C1346736</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/texas-instruments/INA118PB/300978?s=N4IgTCBcDaIJIDkCCBGFAOACgIRAXQF8g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">	
-INA118PB-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">	
-IC INST AMP 1 CIRCUIT 8DIP</t>
-  </si>
-  <si>
-    <t>C1346736</t>
-  </si>
-  <si>
     <t>Manufacturer  part #</t>
-  </si>
-  <si>
-    <t>INA118PB</t>
   </si>
   <si>
     <t>https://www.digikey.com/en/products/detail/texas-instruments/REF2033QDDCRQ1/15926650?s=N4IgTCBcDaIEoFEBiYAMBmdBFAIjgwnFgIwgC6AvkA</t>
@@ -234,9 +214,6 @@
     <t>In Stock?</t>
   </si>
   <si>
-    <t>Yes, only 8 left</t>
-  </si>
-  <si>
     <t>Yes (505 left)</t>
   </si>
   <si>
@@ -457,6 +434,24 @@
   </si>
   <si>
     <t>GCM155R71H104KE02D</t>
+  </si>
+  <si>
+    <t>https://jlcpcb.com/partdetail/TexasInstruments-INA118U2K5/C431293</t>
+  </si>
+  <si>
+    <t>IC INST AMP 1 CIRCUIT 8SOIC</t>
+  </si>
+  <si>
+    <t>296-26056-1-ND</t>
+  </si>
+  <si>
+    <t>INA118U/2K5</t>
+  </si>
+  <si>
+    <t>C431293</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/texas-instruments/INA118U-2K5/2254830?utm_source=chatgpt.com</t>
   </si>
 </sst>
 </file>
@@ -889,7 +884,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>3</v>
@@ -898,40 +893,40 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="J1" s="3"/>
     </row>
     <row r="2" spans="1:10" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>135</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>132</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="H2" s="1" t="s">
-        <v>11</v>
+        <v>133</v>
       </c>
       <c r="I2" s="1">
         <v>4</v>
@@ -940,28 +935,28 @@
     </row>
     <row r="3" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="G3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="I3" s="1">
         <v>1</v>
@@ -969,28 +964,28 @@
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="I4" s="1">
         <v>1</v>
@@ -998,28 +993,28 @@
     </row>
     <row r="5" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="F5" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="I5" s="1">
         <v>1</v>
@@ -1149,14 +1144,14 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{DE32DAC0-DAAB-451D-8121-43B336EB7D31}"/>
-    <hyperlink ref="A2" r:id="rId2" xr:uid="{8E7B69A1-9F16-4CA2-AB60-1B446365ADBD}"/>
-    <hyperlink ref="A3" r:id="rId3" xr:uid="{AD15D0B3-2118-4C28-8A1B-1D076F6B097F}"/>
-    <hyperlink ref="E3" r:id="rId4" xr:uid="{B3C35203-B095-4B55-AAED-6CCED287487A}"/>
-    <hyperlink ref="A4" r:id="rId5" xr:uid="{1023CE1E-0313-4F6A-8A49-4B5FCFAA93EE}"/>
-    <hyperlink ref="A5" r:id="rId6" xr:uid="{DA8D95FB-13FB-4F7F-80F5-8E14E5F2BD50}"/>
-    <hyperlink ref="E5" r:id="rId7" xr:uid="{F163AD94-952E-4351-B375-AD123D63FC34}"/>
-    <hyperlink ref="E4" r:id="rId8" xr:uid="{B6C22098-5BA7-4AEF-AF4E-95C677DF4730}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{AD15D0B3-2118-4C28-8A1B-1D076F6B097F}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{B3C35203-B095-4B55-AAED-6CCED287487A}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{1023CE1E-0313-4F6A-8A49-4B5FCFAA93EE}"/>
+    <hyperlink ref="A5" r:id="rId4" xr:uid="{DA8D95FB-13FB-4F7F-80F5-8E14E5F2BD50}"/>
+    <hyperlink ref="E5" r:id="rId5" xr:uid="{F163AD94-952E-4351-B375-AD123D63FC34}"/>
+    <hyperlink ref="E4" r:id="rId6" xr:uid="{B6C22098-5BA7-4AEF-AF4E-95C677DF4730}"/>
+    <hyperlink ref="E2" r:id="rId7" xr:uid="{49DEC857-9C8A-442E-8FE8-297977B0A3D9}"/>
+    <hyperlink ref="A2" r:id="rId8" xr:uid="{DA248814-7014-41D7-BE88-DC80E3297943}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId9"/>
@@ -1189,7 +1184,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>3</v>
@@ -1198,40 +1193,40 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="J1" s="3"/>
     </row>
     <row r="2" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="I2" s="1">
         <v>16</v>
@@ -1239,28 +1234,28 @@
     </row>
     <row r="3" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="I3" s="1">
         <v>2</v>
@@ -1268,28 +1263,28 @@
     </row>
     <row r="4" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="I4" s="1">
         <v>4</v>
@@ -1297,28 +1292,28 @@
     </row>
     <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>53</v>
-      </c>
       <c r="G5" s="1" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="I5" s="1">
         <v>4</v>
@@ -1326,28 +1321,28 @@
     </row>
     <row r="6" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="I6" s="1">
         <v>4</v>
@@ -1355,28 +1350,28 @@
     </row>
     <row r="7" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="I7" s="1">
         <v>4</v>
@@ -1384,28 +1379,28 @@
     </row>
     <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="I8" s="1">
         <v>2</v>
@@ -1413,28 +1408,28 @@
     </row>
     <row r="9" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="I9" s="1">
         <v>2</v>
@@ -1685,7 +1680,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>3</v>
@@ -1694,39 +1689,39 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>78</v>
       </c>
       <c r="I2" s="1">
         <v>2</v>
@@ -1734,25 +1729,25 @@
     </row>
     <row r="3" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H3" s="1">
         <v>705430004</v>
@@ -1763,25 +1758,25 @@
     </row>
     <row r="4" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H4" s="1">
         <v>705430003</v>
@@ -1792,25 +1787,25 @@
     </row>
     <row r="5" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H5" s="1">
         <v>901361103</v>
@@ -1821,19 +1816,19 @@
     </row>
     <row r="6" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
@@ -1844,19 +1839,19 @@
     </row>
     <row r="7" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -1867,19 +1862,19 @@
     </row>
     <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -1890,28 +1885,28 @@
     </row>
     <row r="9" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="I9" s="1">
         <v>6</v>

</xml_diff>

<commit_message>
finished mcp connector design
</commit_message>
<xml_diff>
--- a/MIB_components.xlsx
+++ b/MIB_components.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arian\Documents\RAMMP\repos\RAMMP-Electronics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA9D20F9-1E93-4824-A66F-427D62F26B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43C9D527-259A-4D70-BBF0-56DB908E81E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{6F4A9416-ED2C-4136-AA62-A972BF68C866}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{6F4A9416-ED2C-4136-AA62-A972BF68C866}"/>
   </bookViews>
   <sheets>
     <sheet name="ICs" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="189">
   <si>
     <t>Digikey link</t>
   </si>
@@ -594,6 +594,24 @@
   </si>
   <si>
     <t>RC0603FR-07931RL</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/keystone-electronics/5003/362668</t>
+  </si>
+  <si>
+    <t>36-5003-ND</t>
+  </si>
+  <si>
+    <t>PC TEST POINT MINIATURE ORANGE</t>
+  </si>
+  <si>
+    <t>Test points</t>
+  </si>
+  <si>
+    <t>https://jlcpcb.com/partdetail/Keystone-5003/C238124?jlc_vid=ElFbA10EEwBaVQECRAILXlEDFVkLVVNXFgcLBlVfQFgxVlNeQFJcU1xRRlddVjtW</t>
+  </si>
+  <si>
+    <t>C238124</t>
   </si>
 </sst>
 </file>
@@ -2392,11 +2410,12 @@
   <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.5546875" customWidth="1"/>
+    <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" customWidth="1"/>
     <col min="3" max="3" width="19.21875" customWidth="1"/>
     <col min="4" max="4" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="31.44140625" customWidth="1"/>
+    <col min="5" max="5" width="39" customWidth="1"/>
+    <col min="6" max="6" width="38.44140625" customWidth="1"/>
     <col min="8" max="8" width="18.77734375" customWidth="1"/>
     <col min="9" max="9" width="13.88671875" customWidth="1"/>
   </cols>
@@ -2459,15 +2478,31 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+    <row r="3" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="1">
+        <v>5003</v>
+      </c>
       <c r="I3" s="1"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -2650,6 +2685,8 @@
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{495BC442-A473-4A63-8A52-76B4B9CEAF2E}"/>
     <hyperlink ref="E2" r:id="rId2" xr:uid="{348AC21B-3EFA-4731-B349-2709FFAF7AC3}"/>
+    <hyperlink ref="A3" r:id="rId3" xr:uid="{B96DC06A-F590-45DF-A2D7-35C2456E0208}"/>
+    <hyperlink ref="E3" r:id="rId4" xr:uid="{4BAF805E-1312-4972-AB0E-B1C6E6C71183}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>